<commit_message>
docs: nouvelle interface README + Details.md, CR d'août
Le README passe en synthèse visuelle (tableaux, graphiques, décisions
attendues en tête) et la version détaillée devient Details.md à la racine.

- README : décisions attendues remontées, chantiers et plan d'actions en
  tableaux, prose déplacée vers les fiches de Details.md
- graphe de maturité d'organisation par périmètre, en remplacement du
  décompte par niveau ; graphe du pipeline d'actions retiré
- CR d'août : atelier DA architectes, atelier skills DACCORD, point
  d'adoption IA produit, suivi Gary
- .gitignore : intermédiaires régénérables des dossiers build/, outillage
  tiers (.tools/) et archives d'artefacts, qui bloquaient le push

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Etat-avancement/Etat-avancement.xlsx
+++ b/Etat-avancement/Etat-avancement.xlsx
@@ -359,7 +359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:L33"/>
+  <dimension ref="A2:L50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="29.67" customWidth="1" style="4" min="2" max="2"/>
@@ -979,7 +979,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Réalisé: - Atelier de formation au développement augmenté À réaliser: - Suivre l'intégration de skills, agents et rules par l'équpe - Rencontre le 6 août pour un atelier d'amélioration des skills</t>
+          <t>Réalisé: - Atelier de formation au développement augmenté (16 juillet) - Mise en commun des system prompts (agents, rules, skills) engagée par l'équipe, premiers skills relus par la mission - Atelier d'amélioration des skills le 6 août: l'équipe a avancé sur ses skills, qui couvrent le changement de version (sensible: il impacte un système de vérification), le changelog, le dev front, le dev back (bonnes pratiques, archi) et le plan d'implémentation - Recommandation: ajouter des skills de tests back et front, l'équipe visant aussi les tests e2e En cours: - Accompagnement individuel pour optimiser les skills et poser les bases de l'orchestration: Sébastien (démarré le 6 août, poursuite courant août), Florian (11 août), Sylvain (début septembre, congés en août) À réaliser: - Obtenir l'accès au code via Rémi pour une analyse et des suggestions - Voir avec Gary l'usage des LLM Irritant remonté: - Forfait trop juste, ce qui pousse l'équipe vers OpenCode</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>En cours: - Adaptation des orchestrations Egapro à Jira</t>
+          <t>En cours: - Adaptation des orchestrations Egapro à Jira À réaliser: - Poser les bases de l'orchestration lors de l'accompagnement individuel d'août (Sébastien, Florian), puis avec Sylvain début septembre</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>À définir</t>
+          <t>À réaliser: - Accompagner Halim sur la génération de tickets intelligibles via MCP, pour des tickets qui génèrent moins d'allers-retours avec les devs (action du point produit du 6 août) - Créneau à caler</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>Réalisé: - Générateurs comparatifs Claude / DeepSeek construits À réaliser: - Atelier de génération de DA avec l'IA le 3 août - Rattacher l'atelier au chantier de démat du DA porté par Igor: structuration du document pas à jour, ressaisie d'information, difficultés de traçage entre versions, stockage et partage sur SharePoint</t>
+          <t>Réalisé: - Générateurs comparatifs Claude / DeepSeek construits - Atelier de génération de DA avec l'IA tenu le 4 août: démonstration de la génération d'un DA depuis un code source, présentation de deux voies d'usage de l'IA sur poste ministère (Claude Code via Bedrock, OpenCode Desktop via Albert). 5 use cases identifiés par les architectes: cohérence des choix techniques entre eux, cohérence vis-à-vis du fonctionnel, conversion de schémas figés en draw.io éditable, conformité des schémas au modèle de DA, écarts entre DA et code réel. Appris au passage: un modèle de DA propre aux applications Atlas existe; deux irritants remontés (ergonomie du DA pénible à remplir, incohérences dans les choix techniques difficiles à percevoir) - Projet expérimental de génération de DA mis à disposition des architectes le 4 août À réaliser: - Les architectes valident / enrichissent la liste de use cases et la priorisent par impact, d'ici au 21 août - Les architectes mappent les parties du DA à leurs sources d'information, d'ici au 21 août - Point de synchronisation pour sélectionner les use cases (et en explorer un si réalisé dans les temps), semaine du 31 août - Rattacher l'atelier au chantier de démat du DA porté par Igor: structuration du document pas à jour, ressaisie d'information, difficultés de traçage entre versions, stockage et partage sur SharePoint</t>
         </is>
       </c>
       <c r="I27" s="8" t="n"/>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>Atelier à positionner au 3 août</t>
+          <t>Réalisé: - Point tenu le 23 juillet avec AWS et Software One, conjointement au cadrage de la voie Bedrock</t>
         </is>
       </c>
       <c r="I28" s="8" t="n"/>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Réalisé: - Igor a identifié les deux voies possibles pour un agent interne sur poste managé, qui ne peut pas installer un harness: soit le packaging de l'application par le centre logiciel, soit une demande de compte administrateur temporaire contresignée par le manager - Côté développeurs, la sécurité s'oriente vers des postes à système libre, avec une VM dédiée à la bureautique. La bureautique n'a pas vocation à tourner sur un environnement aussi ouvert que celui d'un développeur À réaliser: - Rencontrer Céline Liechti, qui saura nous orienter vers les personnes qui gèrent le centre logiciel, pour y faire intégrer les harness cibles - Vérifier les contraintes réseau constatées: npx semble bloqué, HTTP passe</t>
+          <t>Réalisé: - Igor a identifié les deux voies possibles pour un agent interne sur poste managé, qui ne peut pas installer un harness: soit le packaging de l'application par le centre logiciel, soit une demande de compte administrateur temporaire contresignée par le manager - Côté développeurs, la sécurité s'oriente vers des postes à système libre, avec une VM dédiée à la bureautique. La bureautique n'a pas vocation à tourner sur un environnement aussi ouvert que celui d'un développeur - Point produit du 6 août: le centre logiciel peut tolérer des outils restreints à une liste de personnes, et Olivier introduira la mission auprès des personnes qui le gèrent À réaliser: - Rencontrer les personnes du centre logiciel (introduction par Olivier, orientation possible via Céline Liechti) pour y faire intégrer les harness cibles - Vérifier les contraintes réseau constatées: npx semble bloqué, HTTP passe</t>
         </is>
       </c>
     </row>
@@ -1530,6 +1530,271 @@
       <c r="H33" s="8" t="inlineStr">
         <is>
           <t>Réalisé: - Automatisation de la veille du Journal officiel sur les spécialités pharmaceutiques, restituée en newsletter. Le besoin était exprimé "avec de l'IA" et la solution atteint l'objectif sans en avoir besoin - Sabine Lugand est satisfaite de l'outil. MVP réalisé en 3 jours - Passation à Victor Degliame À réaliser (Victor): - Transformer la solution Python en outil utilisable par des personnes qui ne peuvent pas installer Python - Implémenter les évolutions souhaitées par Sabine À réaliser (mission): - Évangéliser les personnes du CEPS que Victor a rencontrées, en capitalisant sur le MVP: 3 jours pour quasi automatiser une newsletter mensuelle. Message: l'IA permet de réaliser des applications rapidement tant que le besoin est clair</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Transverse</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Embarquer la population produit (coachs, PM/PO, RU)</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Réalisé: - Point d'adoption IA du 6 août: la population produit à outiller est hétérogène (coachs, PM/PO, recherche utilisateur) - Les RU craignent d'être remplacés par l'IA et de voir la donnée partir n'importe où: à traiter par des use cases dédiés À réaliser: - Félix formalise et partage les use cases RU et PM/PO - Olivier liste les équipes prioritaires à accompagner sur l'IA - Accompagner les PM sur la génération de tickets intelligibles via MCP: SIRENA, DACCORD, VAO (Halim), BIO2 (Yuna, produit de refonte côté santé, refonte début septembre) - Clarifier l'embarquement de l'équipe de Pierre-Étienne, notamment la synchronisation sur la charte d'usage de l'IA - Regarder OpenWork (suggestion de Félix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Transverse</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Centraliser la documentation fonctionnelle</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>À réaliser: - Sujet jugé prioritaire au point produit du 6 août: un dossier docs, avec des dossiers d'epic contenant la doc - Suggérer à Adrien et Gary de porter le sujet en commun avec le studio produit</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Transverse</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Définir et partager un catalogue de skills communs</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>À réaliser (courant août): - Skill besoin PO: besoin métier, US, tests d'acceptance - Skill plan technique orienté ATDD, prenant en compte les features passées et futures impactées - Skill dev en ATDD (séparation codeur / testeur) - Skill refacto adossé à Sonar - Partager ces skills entre les périmètres accompagnés</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Maturité d'organisation par périmètre (échelle 1 à 5):</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Périmètre</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Niveau (évolution)</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Ce que l'accompagnement a changé</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Egapro</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>3 -&gt; 4</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Les orchestrations tournent en routine et l'organisation est maîtrisée (c'était le chaos, ça ne l'est plus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>DACCORD</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Coaching, skills partagés couvrant cinq domaines, accompagnement individuel engagé. Le niveau 3 se validera quand les skills seront réellement utilisés au quotidien</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>SIRENA</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Usage IA réel mais individuel, sans coordination d'équipe; pas encore d'effet de l'accompagnement (formation mi-août)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>VAO</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Accompagnement à venir (atelier du 8 septembre, tickets avec Halim)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>BIO2</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Nouveau périmètre, accompagnement au lancement de la refonte (début septembre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Architectes</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>1 -&gt; 2</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>L'atelier DA a fait passer la fonction de rien à la découverte: cinq use cases identifiés, priorisation en cours</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Échelle: 1-2 de rien à la découverte de l'IA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>3: des skills utilisés, des use cases IA pratiqués, une organisation perfectible</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>4: des orchestrations, une organisation maîtrisée</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>5: orchestrations, volume de cas d'usage (dev et PM/PO), orga pointue, bonnes pratiques renseignées, vrai craft</t>
         </is>
       </c>
     </row>

</xml_diff>